<commit_message>
generated 50 state vignettes
</commit_message>
<xml_diff>
--- a/AHR_data 28th.xlsx
+++ b/AHR_data 28th.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tn/Desktop/REASON/AHR_50states/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E266698-91C3-394D-9E97-AF7EEF6FB51D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7170B722-8D77-6B44-842E-059E0B8B54E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="5500" windowWidth="30240" windowHeight="14200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="5500" windowWidth="44560" windowHeight="16200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AHR Data" sheetId="1" r:id="rId1"/>
@@ -14228,7 +14228,7 @@
         <v>8</v>
       </c>
       <c r="Q45" s="3">
-        <v>41.327527577092397</v>
+        <v>12.499602169524961</v>
       </c>
     </row>
     <row r="46" spans="1:17" x14ac:dyDescent="0.2">
@@ -14281,7 +14281,7 @@
         <v>44</v>
       </c>
       <c r="Q46" s="3">
-        <v>12.499602169524961</v>
+        <v>9.1521387309594004</v>
       </c>
     </row>
     <row r="47" spans="1:17" x14ac:dyDescent="0.2">
@@ -14334,7 +14334,7 @@
         <v>4</v>
       </c>
       <c r="Q47" s="3">
-        <v>9.1521387309594004</v>
+        <v>39.178114774360743</v>
       </c>
     </row>
     <row r="48" spans="1:17" x14ac:dyDescent="0.2">
@@ -14387,7 +14387,7 @@
         <v>47</v>
       </c>
       <c r="Q48" s="3">
-        <v>39.178114774360743</v>
+        <v>27.761212395925181</v>
       </c>
     </row>
     <row r="49" spans="1:17" x14ac:dyDescent="0.2">
@@ -14440,7 +14440,7 @@
         <v>33</v>
       </c>
       <c r="Q49" s="3">
-        <v>27.761212395925181</v>
+        <v>9.2002820844321178</v>
       </c>
     </row>
     <row r="50" spans="1:17" x14ac:dyDescent="0.2">
@@ -14493,7 +14493,7 @@
         <v>26</v>
       </c>
       <c r="Q50" s="3">
-        <v>9.2002820844321178</v>
+        <v>16.718221641439211</v>
       </c>
     </row>
     <row r="51" spans="1:17" x14ac:dyDescent="0.2">
@@ -14546,7 +14546,7 @@
         <v>12</v>
       </c>
       <c r="Q51" s="3">
-        <v>16.718221641439211</v>
+        <v>7.7436829870209873</v>
       </c>
     </row>
   </sheetData>

</xml_diff>